<commit_message>
Add Selenium web E2E test suite and Excel report
</commit_message>
<xml_diff>
--- a/testing/reports/Selenium_Web_E2E_Test_Report.xlsx
+++ b/testing/reports/Selenium_Web_E2E_Test_Report.xlsx
@@ -26,7 +26,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>7/28/2026, 1:52:56 PM</t>
+    <t>7/30/2026, 10:11:49 AM</t>
   </si>
   <si>
     <t>Total Test Cases Executed</t>
@@ -47,7 +47,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>128.79 seconds</t>
+    <t>98.77 seconds</t>
   </si>
   <si>
     <t>Suite Name</t>
@@ -86,7 +86,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-07-28T08:20:52.756Z</t>
+    <t>2026-07-30T04:40:26.541Z</t>
   </si>
   <si>
     <t/>
@@ -101,7 +101,7 @@
     <t>Validate Form Validation for Invalid Credentials</t>
   </si>
   <si>
-    <t>2026-07-28T08:21:23.403Z</t>
+    <t>2026-07-30T04:40:37.036Z</t>
   </si>
   <si>
     <t>Invalid credentials input handled gracefully by authentication state.</t>
@@ -113,7 +113,7 @@
     <t>Validate User Login with Valid Credentials</t>
   </si>
   <si>
-    <t>2026-07-28T08:21:53.911Z</t>
+    <t>2026-07-30T04:40:47.450Z</t>
   </si>
   <si>
     <t>User login payload submitted and processed by Supabase auth.</t>
@@ -128,7 +128,7 @@
     <t>Navigate to Session History Tab</t>
   </si>
   <si>
-    <t>2026-07-28T08:22:03.976Z</t>
+    <t>2026-07-30T04:40:57.485Z</t>
   </si>
   <si>
     <t>Switched to Session History tab successfully.</t>
@@ -140,7 +140,7 @@
     <t>Navigate to User Profile Screen</t>
   </si>
   <si>
-    <t>2026-07-28T08:22:14.059Z</t>
+    <t>2026-07-30T04:41:07.579Z</t>
   </si>
   <si>
     <t>Switched to User Profile tab successfully.</t>
@@ -155,7 +155,7 @@
     <t>Open Camera Session Recording Screen</t>
   </si>
   <si>
-    <t>2026-07-28T08:22:24.104Z</t>
+    <t>2026-07-30T04:41:17.625Z</t>
   </si>
   <si>
     <t>Camera viewport opened with media permission handling.</t>
@@ -167,7 +167,7 @@
     <t>Record Video &amp; Submit for AI Posture Analysis</t>
   </si>
   <si>
-    <t>2026-07-28T08:22:56.369Z</t>
+    <t>2026-07-30T04:41:49.844Z</t>
   </si>
   <si>
     <t>Video recorded and payload sent to FastAPI /analyze endpoint.</t>
@@ -741,7 +741,7 @@
         <v>23</v>
       </c>
       <c r="E2">
-        <v>5184</v>
+        <v>15466</v>
       </c>
       <c r="F2" t="s">
         <v>24</v>
@@ -767,7 +767,7 @@
         <v>23</v>
       </c>
       <c r="E3">
-        <v>30646</v>
+        <v>10494</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -793,7 +793,7 @@
         <v>23</v>
       </c>
       <c r="E4">
-        <v>30508</v>
+        <v>10414</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -819,7 +819,7 @@
         <v>23</v>
       </c>
       <c r="E5">
-        <v>10064</v>
+        <v>10034</v>
       </c>
       <c r="F5" t="s">
         <v>38</v>
@@ -845,7 +845,7 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>10083</v>
+        <v>10094</v>
       </c>
       <c r="F6" t="s">
         <v>42</v>
@@ -871,7 +871,7 @@
         <v>23</v>
       </c>
       <c r="E7">
-        <v>10044</v>
+        <v>10045</v>
       </c>
       <c r="F7" t="s">
         <v>47</v>
@@ -897,7 +897,7 @@
         <v>23</v>
       </c>
       <c r="E8">
-        <v>32264</v>
+        <v>32218</v>
       </c>
       <c r="F8" t="s">
         <v>51</v>

</xml_diff>